<commit_message>
fix(ci): sanitize GitHub Action versions to canonical v4/v5/v2 across all workflows
</commit_message>
<xml_diff>
--- a/reports/coordination/AGENT_OPERATING_OPTIONS.xlsx
+++ b/reports/coordination/AGENT_OPERATING_OPTIONS.xlsx
@@ -887,7 +887,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-25T13:30:05.855013+00:00</t>
+          <t>2026-08-29T11:11:00.082029+00:00</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>719566d23fd9aeb783a72fcec9493557f783781f</t>
+          <t>01a4592f4c68c120a26b4fd955d1aff655b82e33</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2/7</t>
+          <t>3/7</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AUTH_OK v319</t>
+          <t>AUTH_OK v323</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>serving=719566d (compare origin/main in session)</t>
+          <t>serving=01a4592 (compare origin/main in session)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>healthy=False http=200</t>
+          <t>healthy=True http=200</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>connected=True auth=AUTH_OK v=319</t>
+          <t>connected=True auth=AUTH_OK v=323</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>holdings=404 funds=404</t>
+          <t>holdings=200 funds=200</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>pass=False</t>
+          <t>pass=True</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>gates=2/7 trade_ready=False</t>
+          <t>gates=3/7 trade_ready=False</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">

</xml_diff>